<commit_message>
Finished layout of wpa
can translate morse to english and vice versa. need to translate other languages and code buttons
</commit_message>
<xml_diff>
--- a/Gantt Chart.xlsx
+++ b/Gantt Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveplymouthac-my.sharepoint.com/personal/kayleigh_soane_students_plymouth_ac_uk/Documents/Github Repositories/COMP1004ComputingProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:11_{BCF52E15-7D68-4602-832E-A696C3A242EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EEBDB17-A28F-4932-AADA-CA1581FE6C9F}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="13_ncr:11_{BCF52E15-7D68-4602-832E-A696C3A242EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E38F028-4579-4AE6-B815-998E34D5BF30}"/>
   <bookViews>
-    <workbookView xWindow="2290" yWindow="0" windowWidth="14400" windowHeight="12090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>Project Planner</t>
   </si>
@@ -48,12 +48,6 @@
     <t>ACTIVITY</t>
   </si>
   <si>
-    <t>Activity 16</t>
-  </si>
-  <si>
-    <t>Activity 17</t>
-  </si>
-  <si>
     <t>Activity 18</t>
   </si>
   <si>
@@ -73,12 +67,6 @@
   </si>
   <si>
     <t>Activity 24</t>
-  </si>
-  <si>
-    <t>Activity 25</t>
-  </si>
-  <si>
-    <t>Activity 26</t>
   </si>
   <si>
     <r>
@@ -210,28 +198,37 @@
     <t>Develop API integration</t>
   </si>
   <si>
-    <t>Create text input system</t>
-  </si>
-  <si>
     <t>Create buttons for languages</t>
   </si>
   <si>
-    <t>Create text output system</t>
-  </si>
-  <si>
     <t>Create morse code library</t>
   </si>
   <si>
     <t>Create system to translate letters to morse</t>
   </si>
   <si>
-    <t>Get buttons to identify input language</t>
-  </si>
-  <si>
-    <t>Use buttons to decide what language to output</t>
-  </si>
-  <si>
     <t>If text too big for box, can scroll down inside box</t>
+  </si>
+  <si>
+    <t>Create text output box</t>
+  </si>
+  <si>
+    <t>Create text input box</t>
+  </si>
+  <si>
+    <t>Automcatically detect input language</t>
+  </si>
+  <si>
+    <t>Use dropdown to select input</t>
+  </si>
+  <si>
+    <t>Use dropdown to select output</t>
+  </si>
+  <si>
+    <t>Make JS code to translate morse code</t>
+  </si>
+  <si>
+    <t>Text to speech</t>
   </si>
 </sst>
 </file>
@@ -1081,21 +1078,21 @@
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="25" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C2" s="25"/>
       <c r="D2" s="25"/>
       <c r="E2" s="25"/>
       <c r="F2" s="25"/>
       <c r="G2" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H2" s="14">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J2" s="15"/>
       <c r="K2" s="31" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
@@ -1103,21 +1100,21 @@
       <c r="O2" s="33"/>
       <c r="P2" s="16"/>
       <c r="Q2" s="31" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="R2" s="34"/>
       <c r="S2" s="34"/>
       <c r="T2" s="33"/>
       <c r="U2" s="17"/>
       <c r="V2" s="23" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="W2" s="24"/>
       <c r="X2" s="24"/>
       <c r="Y2" s="35"/>
       <c r="Z2" s="18"/>
       <c r="AA2" s="23" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="AB2" s="24"/>
       <c r="AC2" s="24"/>
@@ -1127,7 +1124,7 @@
       <c r="AG2" s="35"/>
       <c r="AH2" s="19"/>
       <c r="AI2" s="23" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="AJ2" s="24"/>
       <c r="AK2" s="24"/>
@@ -1142,19 +1139,19 @@
         <v>2</v>
       </c>
       <c r="C3" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="30" t="s">
         <v>18</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>22</v>
       </c>
       <c r="H3" s="20" t="s">
         <v>1</v>
@@ -1368,57 +1365,57 @@
       </c>
     </row>
     <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="6">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6">
-        <v>1</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="21" t="s">
-        <v>27</v>
-      </c>
       <c r="C6" s="6">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D6" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F6" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="22" t="s">
-        <v>28</v>
+      <c r="B7" s="21" t="s">
+        <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
@@ -1429,13 +1426,13 @@
     </row>
     <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B8" s="21" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="C8" s="6">
         <v>0</v>
       </c>
       <c r="D8" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="6">
         <v>0</v>
@@ -1449,13 +1446,13 @@
     </row>
     <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B9" s="22" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="C9" s="6">
         <v>0</v>
       </c>
       <c r="D9" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6">
         <v>0</v>
@@ -1469,13 +1466,13 @@
     </row>
     <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B10" s="21" t="s">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="C10" s="6">
         <v>0</v>
       </c>
       <c r="D10" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6">
         <v>0</v>
@@ -1489,13 +1486,13 @@
     </row>
     <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B11" s="22" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="C11" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="6">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E11" s="6">
         <v>0</v>
@@ -1509,7 +1506,7 @@
     </row>
     <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B12" s="21" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C12" s="6">
         <v>0</v>
@@ -1529,13 +1526,13 @@
     </row>
     <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B13" s="22" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="C13" s="6">
         <v>0</v>
       </c>
       <c r="D13" s="6">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E13" s="6">
         <v>0</v>
@@ -1549,13 +1546,13 @@
     </row>
     <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B14" s="21" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="C14" s="6">
         <v>0</v>
       </c>
       <c r="D14" s="6">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E14" s="6">
         <v>0</v>
@@ -1568,17 +1565,15 @@
       </c>
     </row>
     <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="8">
+      <c r="B15" s="22"/>
+      <c r="C15" s="6">
         <v>0</v>
       </c>
       <c r="D15" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E15" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="6">
         <v>0</v>
@@ -1588,77 +1583,77 @@
       </c>
     </row>
     <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="21" t="s">
-        <v>37</v>
+      <c r="B16" s="22" t="s">
+        <v>22</v>
       </c>
       <c r="C16" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E16" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="22" t="s">
-        <v>38</v>
+      <c r="B17" s="21" t="s">
+        <v>23</v>
       </c>
       <c r="C17" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="6">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E17" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="21" t="s">
-        <v>39</v>
+      <c r="B18" s="22" t="s">
+        <v>24</v>
       </c>
       <c r="C18" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E18" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B19" s="22" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="C19" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E19" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="6">
         <v>0</v>
@@ -1669,190 +1664,190 @@
     </row>
     <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B20" s="21" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="C20" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D20" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E20" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B21" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="6">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="C21" s="8">
+        <v>3</v>
       </c>
       <c r="D21" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E21" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F21" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B22" s="21" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C22" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D22" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E22" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F22" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G22" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B23" s="22" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="C23" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D23" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E23" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F23" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B24" s="21" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C24" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D24" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E24" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B25" s="22" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="C25" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D25" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E25" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F25" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B26" s="21" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="C26" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D26" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E26" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F26" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B27" s="22" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C27" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D27" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E27" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F27" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="21" t="s">
-        <v>11</v>
+      <c r="B28" s="22" t="s">
+        <v>38</v>
       </c>
       <c r="C28" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D28" s="6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E28" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F28" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="22" t="s">
-        <v>12</v>
+      <c r="B29" s="21" t="s">
+        <v>28</v>
       </c>
       <c r="C29" s="6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D29" s="6">
         <v>0</v>
@@ -1869,10 +1864,10 @@
     </row>
     <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B30" s="21" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="C30" s="6">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="D30" s="6">
         <v>0</v>
@@ -1888,6 +1883,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:BO30">
+    <sortCondition ref="C5:C30"/>
+  </sortState>
   <mergeCells count="12">
     <mergeCell ref="AI2:AP2"/>
     <mergeCell ref="B2:F2"/>

</xml_diff>

<commit_message>
Upload for leader meeting
</commit_message>
<xml_diff>
--- a/Gantt Chart.xlsx
+++ b/Gantt Chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveplymouthac-my.sharepoint.com/personal/kayleigh_soane_students_plymouth_ac_uk/Documents/Github Repositories/COMP1004ComputingProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="13_ncr:11_{BCF52E15-7D68-4602-832E-A696C3A242EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E38F028-4579-4AE6-B815-998E34D5BF30}"/>
+  <xr:revisionPtr revIDLastSave="281" documentId="13_ncr:11_{BCF52E15-7D68-4602-832E-A696C3A242EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C58EB54-D7DA-4384-88A2-E3E60C4CBC21}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Project Planner</t>
   </si>
@@ -46,27 +46,6 @@
   </si>
   <si>
     <t>ACTIVITY</t>
-  </si>
-  <si>
-    <t>Activity 18</t>
-  </si>
-  <si>
-    <t>Activity 19</t>
-  </si>
-  <si>
-    <t>Activity 20</t>
-  </si>
-  <si>
-    <t>Activity 21</t>
-  </si>
-  <si>
-    <t>Activity 22</t>
-  </si>
-  <si>
-    <t>Activity 23</t>
-  </si>
-  <si>
-    <t>Activity 24</t>
   </si>
   <si>
     <r>
@@ -180,24 +159,12 @@
     <t>Create UI plan</t>
   </si>
   <si>
-    <t>Design UI</t>
-  </si>
-  <si>
     <t>Make text boxes</t>
   </si>
   <si>
-    <t>Create light and dark themes</t>
-  </si>
-  <si>
-    <t>Create buttons for theme</t>
-  </si>
-  <si>
     <t>Research API</t>
   </si>
   <si>
-    <t>Develop API integration</t>
-  </si>
-  <si>
     <t>Create buttons for languages</t>
   </si>
   <si>
@@ -228,7 +195,43 @@
     <t>Make JS code to translate morse code</t>
   </si>
   <si>
-    <t>Text to speech</t>
+    <t>Create buttons for copy, text to speech, about etc</t>
+  </si>
+  <si>
+    <t>Create dropdown for theme</t>
+  </si>
+  <si>
+    <t>Link an about page with button</t>
+  </si>
+  <si>
+    <t>Make code to reverse dropdown values</t>
+  </si>
+  <si>
+    <t>Link github page</t>
+  </si>
+  <si>
+    <t>mid-project review</t>
+  </si>
+  <si>
+    <t>Activity 21</t>
+  </si>
+  <si>
+    <t>Make translation occur upon input - no button</t>
+  </si>
+  <si>
+    <t>Design UI layout</t>
+  </si>
+  <si>
+    <t>Secure API key in backend proxy server?</t>
+  </si>
+  <si>
+    <t>integrate api translator</t>
+  </si>
+  <si>
+    <t>make page themes</t>
+  </si>
+  <si>
+    <t>code to make theme selector work</t>
   </si>
 </sst>
 </file>
@@ -336,7 +339,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -381,12 +384,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -553,15 +550,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="4">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -598,12 +586,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="11">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="2" applyFont="1" applyFill="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -642,6 +624,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -1067,122 +1064,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.25">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
+      <c r="B2" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
       <c r="G2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="11">
+        <v>18</v>
+      </c>
+      <c r="J2" s="12"/>
+      <c r="K2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="14">
-        <v>15</v>
-      </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="31" t="s">
-        <v>19</v>
-      </c>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
-      <c r="T2" s="33"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="23" t="s">
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="R2" s="29"/>
+      <c r="S2" s="29"/>
+      <c r="T2" s="28"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="W2" s="19"/>
+      <c r="X2" s="19"/>
+      <c r="Y2" s="30"/>
+      <c r="Z2" s="15"/>
+      <c r="AA2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB2" s="19"/>
+      <c r="AC2" s="19"/>
+      <c r="AD2" s="19"/>
+      <c r="AE2" s="19"/>
+      <c r="AF2" s="19"/>
+      <c r="AG2" s="30"/>
+      <c r="AH2" s="16"/>
+      <c r="AI2" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="AJ2" s="19"/>
+      <c r="AK2" s="19"/>
+      <c r="AL2" s="19"/>
+      <c r="AM2" s="19"/>
+      <c r="AN2" s="19"/>
+      <c r="AO2" s="19"/>
+      <c r="AP2" s="19"/>
+    </row>
+    <row r="3" spans="2:67" s="8" customFormat="1" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="W2" s="24"/>
-      <c r="X2" s="24"/>
-      <c r="Y2" s="35"/>
-      <c r="Z2" s="18"/>
-      <c r="AA2" s="23" t="s">
+      <c r="G3" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="AB2" s="24"/>
-      <c r="AC2" s="24"/>
-      <c r="AD2" s="24"/>
-      <c r="AE2" s="24"/>
-      <c r="AF2" s="24"/>
-      <c r="AG2" s="35"/>
-      <c r="AH2" s="19"/>
-      <c r="AI2" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="AJ2" s="24"/>
-      <c r="AK2" s="24"/>
-      <c r="AL2" s="24"/>
-      <c r="AM2" s="24"/>
-      <c r="AN2" s="24"/>
-      <c r="AO2" s="24"/>
-      <c r="AP2" s="24"/>
-    </row>
-    <row r="3" spans="2:67" s="11" customFormat="1" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="26" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="I3" s="9"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10"/>
-      <c r="W3" s="10"/>
-      <c r="X3" s="10"/>
-      <c r="Y3" s="10"/>
-      <c r="Z3" s="10"/>
-      <c r="AA3" s="10"/>
+      <c r="H3" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="6"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="7"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="27"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -1364,527 +1361,529 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="21" t="s">
+    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="32">
+        <v>0</v>
+      </c>
+      <c r="D5" s="32">
+        <v>0</v>
+      </c>
+      <c r="E5" s="32">
+        <v>0</v>
+      </c>
+      <c r="F5" s="32">
+        <v>0</v>
+      </c>
+      <c r="G5" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="32">
+        <v>21</v>
+      </c>
+      <c r="D6" s="32">
+        <v>2</v>
+      </c>
+      <c r="E6" s="32">
+        <v>0</v>
+      </c>
+      <c r="F6" s="32">
+        <v>0</v>
+      </c>
+      <c r="G6" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="32">
+        <v>20</v>
+      </c>
+      <c r="D7" s="32">
+        <v>1</v>
+      </c>
+      <c r="E7" s="32">
+        <v>18</v>
+      </c>
+      <c r="F7" s="32">
+        <v>0</v>
+      </c>
+      <c r="G7" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="32">
         <v>25</v>
       </c>
-      <c r="C5" s="6">
+      <c r="D8" s="32">
+        <v>5</v>
+      </c>
+      <c r="E8" s="32">
         <v>0</v>
       </c>
-      <c r="D5" s="6">
-        <v>1</v>
-      </c>
-      <c r="E5" s="6">
+      <c r="F8" s="32">
         <v>0</v>
       </c>
-      <c r="F5" s="6">
+      <c r="G8" s="33">
         <v>0</v>
       </c>
-      <c r="G5" s="7">
+    </row>
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="32">
+        <v>26</v>
+      </c>
+      <c r="D9" s="32">
+        <v>7</v>
+      </c>
+      <c r="E9" s="32">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="22" t="s">
+      <c r="F9" s="32">
+        <v>0</v>
+      </c>
+      <c r="G9" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="32">
+        <v>1</v>
+      </c>
+      <c r="D10" s="32">
+        <v>1</v>
+      </c>
+      <c r="E10" s="32">
+        <v>1</v>
+      </c>
+      <c r="F10" s="32">
+        <v>1</v>
+      </c>
+      <c r="G10" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="32">
+        <v>1</v>
+      </c>
+      <c r="D11" s="32">
+        <v>4</v>
+      </c>
+      <c r="E11" s="32">
+        <v>1</v>
+      </c>
+      <c r="F11" s="32">
+        <v>17</v>
+      </c>
+      <c r="G11" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="32">
+        <v>1</v>
+      </c>
+      <c r="D12" s="32">
+        <v>2</v>
+      </c>
+      <c r="E12" s="32">
+        <v>1</v>
+      </c>
+      <c r="F12" s="32">
+        <v>2</v>
+      </c>
+      <c r="G12" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="32">
+        <v>1</v>
+      </c>
+      <c r="D13" s="32">
+        <v>7</v>
+      </c>
+      <c r="E13" s="32">
+        <v>1</v>
+      </c>
+      <c r="F13" s="32">
+        <v>18</v>
+      </c>
+      <c r="G13" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="32">
+        <v>2</v>
+      </c>
+      <c r="D14" s="32">
+        <v>2</v>
+      </c>
+      <c r="E14" s="32">
+        <v>2</v>
+      </c>
+      <c r="F14" s="32">
+        <v>1</v>
+      </c>
+      <c r="G14" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="34">
+        <v>3</v>
+      </c>
+      <c r="D15" s="32">
+        <v>3</v>
+      </c>
+      <c r="E15" s="32">
+        <v>3</v>
+      </c>
+      <c r="F15" s="32">
+        <v>1</v>
+      </c>
+      <c r="G15" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="32">
+        <v>4</v>
+      </c>
+      <c r="D16" s="32">
+        <v>3</v>
+      </c>
+      <c r="E16" s="32">
+        <v>3</v>
+      </c>
+      <c r="F16" s="32">
+        <v>1</v>
+      </c>
+      <c r="G16" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="32">
+        <v>4</v>
+      </c>
+      <c r="D17" s="32">
+        <v>3</v>
+      </c>
+      <c r="E17" s="32">
+        <v>3</v>
+      </c>
+      <c r="F17" s="32">
+        <v>1</v>
+      </c>
+      <c r="G17" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="32">
+        <v>4</v>
+      </c>
+      <c r="D18" s="32">
+        <v>2</v>
+      </c>
+      <c r="E18" s="32">
+        <v>3</v>
+      </c>
+      <c r="F18" s="32">
+        <v>1</v>
+      </c>
+      <c r="G18" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="32">
+        <v>5</v>
+      </c>
+      <c r="D19" s="32">
+        <v>5</v>
+      </c>
+      <c r="E19" s="32">
+        <v>3</v>
+      </c>
+      <c r="F19" s="32">
+        <v>4</v>
+      </c>
+      <c r="G19" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="32">
+        <v>3</v>
+      </c>
+      <c r="D20" s="32">
+        <v>3</v>
+      </c>
+      <c r="E20" s="32">
+        <v>4</v>
+      </c>
+      <c r="F20" s="32">
+        <v>2</v>
+      </c>
+      <c r="G20" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="32">
+        <v>4</v>
+      </c>
+      <c r="D21" s="32">
+        <v>4</v>
+      </c>
+      <c r="E21" s="32">
+        <v>4</v>
+      </c>
+      <c r="F21" s="32">
+        <v>1</v>
+      </c>
+      <c r="G21" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="6">
-        <v>20</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="C22" s="32">
+        <v>4</v>
+      </c>
+      <c r="D22" s="32">
+        <v>4</v>
+      </c>
+      <c r="E22" s="32">
+        <v>5</v>
+      </c>
+      <c r="F22" s="32">
         <v>2</v>
       </c>
-      <c r="E6" s="6">
+      <c r="G22" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="32">
+        <v>7</v>
+      </c>
+      <c r="D23" s="32">
+        <v>2</v>
+      </c>
+      <c r="E23" s="32">
         <v>10</v>
       </c>
-      <c r="F6" s="6">
-        <v>1</v>
-      </c>
-      <c r="G6" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="21" t="s">
+      <c r="F23" s="32">
+        <v>1</v>
+      </c>
+      <c r="G23" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="32">
+        <v>21</v>
+      </c>
+      <c r="D24" s="32">
+        <v>2</v>
+      </c>
+      <c r="E24" s="32">
+        <v>10</v>
+      </c>
+      <c r="F24" s="32">
+        <v>1</v>
+      </c>
+      <c r="G24" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="32">
+        <v>11</v>
+      </c>
+      <c r="D25" s="32">
+        <v>1</v>
+      </c>
+      <c r="E25" s="32">
+        <v>11</v>
+      </c>
+      <c r="F25" s="32">
+        <v>1</v>
+      </c>
+      <c r="G25" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="32">
+        <v>15</v>
+      </c>
+      <c r="D26" s="32">
+        <v>3</v>
+      </c>
+      <c r="E26" s="32">
+        <v>15</v>
+      </c>
+      <c r="F26" s="32">
+        <v>3</v>
+      </c>
+      <c r="G26" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="32">
+        <v>11</v>
+      </c>
+      <c r="D27" s="32">
+        <v>2</v>
+      </c>
+      <c r="E27" s="32">
+        <v>16</v>
+      </c>
+      <c r="F27" s="32">
+        <v>1</v>
+      </c>
+      <c r="G27" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="32">
+        <v>12</v>
+      </c>
+      <c r="D28" s="32">
+        <v>2</v>
+      </c>
+      <c r="E28" s="32">
+        <v>16</v>
+      </c>
+      <c r="F28" s="32">
+        <v>1</v>
+      </c>
+      <c r="G28" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="6">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6">
-        <v>0</v>
-      </c>
-      <c r="G7" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="6">
-        <v>0</v>
-      </c>
-      <c r="D8" s="6">
-        <v>0</v>
-      </c>
-      <c r="E8" s="6">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="6">
-        <v>0</v>
-      </c>
-      <c r="D9" s="6">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6">
-        <v>0</v>
-      </c>
-      <c r="G9" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="21" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="6">
-        <v>0</v>
-      </c>
-      <c r="D10" s="6">
-        <v>0</v>
-      </c>
-      <c r="E10" s="6">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="6">
-        <v>0</v>
-      </c>
-      <c r="D11" s="6">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6">
-        <v>0</v>
-      </c>
-      <c r="F11" s="6">
-        <v>0</v>
-      </c>
-      <c r="G11" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="21" t="s">
+      <c r="C29" s="32">
+        <v>22</v>
+      </c>
+      <c r="D29" s="32">
+        <v>2</v>
+      </c>
+      <c r="E29" s="32">
+        <v>16</v>
+      </c>
+      <c r="F29" s="32">
+        <v>1</v>
+      </c>
+      <c r="G29" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="32">
         <v>7</v>
       </c>
-      <c r="C12" s="6">
-        <v>0</v>
-      </c>
-      <c r="D12" s="6">
-        <v>0</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="6">
-        <v>0</v>
-      </c>
-      <c r="D13" s="6">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6">
-        <v>0</v>
-      </c>
-      <c r="G13" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="6">
-        <v>0</v>
-      </c>
-      <c r="D14" s="6">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="22"/>
-      <c r="C15" s="6">
-        <v>0</v>
-      </c>
-      <c r="D15" s="6">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6">
-        <v>0</v>
-      </c>
-      <c r="G15" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" s="6">
-        <v>1</v>
-      </c>
-      <c r="D16" s="6">
-        <v>1</v>
-      </c>
-      <c r="E16" s="6">
-        <v>1</v>
-      </c>
-      <c r="F16" s="6">
-        <v>1</v>
-      </c>
-      <c r="G16" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="6">
-        <v>1</v>
-      </c>
-      <c r="D17" s="6">
-        <v>4</v>
-      </c>
-      <c r="E17" s="6">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6">
+      <c r="D30" s="32">
+        <v>7</v>
+      </c>
+      <c r="E30" s="32">
+        <v>17</v>
+      </c>
+      <c r="F30" s="32">
         <v>2</v>
       </c>
-      <c r="G17" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" s="6">
-        <v>1</v>
-      </c>
-      <c r="D18" s="6">
-        <v>2</v>
-      </c>
-      <c r="E18" s="6">
-        <v>1</v>
-      </c>
-      <c r="F18" s="6">
-        <v>2</v>
-      </c>
-      <c r="G18" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="6">
-        <v>1</v>
-      </c>
-      <c r="D19" s="6">
-        <v>7</v>
-      </c>
-      <c r="E19" s="6">
-        <v>1</v>
-      </c>
-      <c r="F19" s="6">
-        <v>0</v>
-      </c>
-      <c r="G19" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="6">
-        <v>2</v>
-      </c>
-      <c r="D20" s="6">
-        <v>2</v>
-      </c>
-      <c r="E20" s="6">
-        <v>2</v>
-      </c>
-      <c r="F20" s="6">
-        <v>1</v>
-      </c>
-      <c r="G20" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="8">
-        <v>3</v>
-      </c>
-      <c r="D21" s="6">
-        <v>3</v>
-      </c>
-      <c r="E21" s="6">
-        <v>3</v>
-      </c>
-      <c r="F21" s="6">
-        <v>1</v>
-      </c>
-      <c r="G21" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="6">
-        <v>3</v>
-      </c>
-      <c r="D22" s="6">
-        <v>3</v>
-      </c>
-      <c r="E22" s="6">
-        <v>4</v>
-      </c>
-      <c r="F22" s="6">
-        <v>2</v>
-      </c>
-      <c r="G22" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" s="6">
-        <v>4</v>
-      </c>
-      <c r="D23" s="6">
-        <v>3</v>
-      </c>
-      <c r="E23" s="6">
-        <v>3</v>
-      </c>
-      <c r="F23" s="6">
-        <v>1</v>
-      </c>
-      <c r="G23" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" s="6">
-        <v>4</v>
-      </c>
-      <c r="D24" s="6">
-        <v>3</v>
-      </c>
-      <c r="E24" s="6">
-        <v>3</v>
-      </c>
-      <c r="F24" s="6">
-        <v>1</v>
-      </c>
-      <c r="G24" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" s="6">
-        <v>4</v>
-      </c>
-      <c r="D25" s="6">
-        <v>4</v>
-      </c>
-      <c r="E25" s="6">
-        <v>4</v>
-      </c>
-      <c r="F25" s="6">
-        <v>1</v>
-      </c>
-      <c r="G25" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="6">
-        <v>4</v>
-      </c>
-      <c r="D26" s="6">
-        <v>4</v>
-      </c>
-      <c r="E26" s="6">
-        <v>5</v>
-      </c>
-      <c r="F26" s="6">
-        <v>2</v>
-      </c>
-      <c r="G26" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B27" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="6">
-        <v>4</v>
-      </c>
-      <c r="D27" s="6">
-        <v>2</v>
-      </c>
-      <c r="E27" s="6">
-        <v>3</v>
-      </c>
-      <c r="F27" s="6">
-        <v>1</v>
-      </c>
-      <c r="G27" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="6">
-        <v>5</v>
-      </c>
-      <c r="D28" s="6">
-        <v>5</v>
-      </c>
-      <c r="E28" s="6">
-        <v>3</v>
-      </c>
-      <c r="F28" s="6">
-        <v>2</v>
-      </c>
-      <c r="G28" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="C29" s="6">
-        <v>7</v>
-      </c>
-      <c r="D29" s="6">
-        <v>0</v>
-      </c>
-      <c r="E29" s="6">
-        <v>0</v>
-      </c>
-      <c r="F29" s="6">
-        <v>0</v>
-      </c>
-      <c r="G29" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="6">
-        <v>28</v>
-      </c>
-      <c r="D30" s="6">
-        <v>0</v>
-      </c>
-      <c r="E30" s="6">
-        <v>0</v>
-      </c>
-      <c r="F30" s="6">
-        <v>0</v>
-      </c>
-      <c r="G30" s="7">
-        <v>0</v>
+      <c r="G30" s="33">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:BO30">
-    <sortCondition ref="C5:C30"/>
+    <sortCondition ref="E5:E30"/>
   </sortState>
   <mergeCells count="12">
     <mergeCell ref="AI2:AP2"/>

</xml_diff>

<commit_message>
Upload for stand-up meeting
</commit_message>
<xml_diff>
--- a/Gantt Chart.xlsx
+++ b/Gantt Chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveplymouthac-my.sharepoint.com/personal/kayleigh_soane_students_plymouth_ac_uk/Documents/Github Repositories/COMP1004ComputingProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="281" documentId="13_ncr:11_{BCF52E15-7D68-4602-832E-A696C3A242EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C58EB54-D7DA-4384-88A2-E3E60C4CBC21}"/>
+  <xr:revisionPtr revIDLastSave="290" documentId="13_ncr:11_{BCF52E15-7D68-4602-832E-A696C3A242EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{915F8D3C-4AAD-4082-8D84-096D8B0B6697}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -586,6 +586,21 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="11">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -624,21 +639,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -1060,7 +1060,20 @@
     <col min="2" max="2" width="24.83203125" style="2" customWidth="1"/>
     <col min="3" max="6" width="11.58203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="15.58203125" style="4" customWidth="1"/>
-    <col min="8" max="27" width="2.75" style="1"/>
+    <col min="8" max="8" width="3.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16" width="2.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="3.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="26" width="3.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="4.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="37" width="4.08203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="39" max="47" width="4.08203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="49" max="57" width="4.08203125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="67" width="4.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.25">
@@ -1074,80 +1087,80 @@
       <c r="G1" s="9"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
       <c r="G2" s="5" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J2" s="12"/>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="28"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="33"/>
       <c r="P2" s="13"/>
-      <c r="Q2" s="26" t="s">
+      <c r="Q2" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="R2" s="29"/>
-      <c r="S2" s="29"/>
-      <c r="T2" s="28"/>
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
+      <c r="T2" s="33"/>
       <c r="U2" s="14"/>
-      <c r="V2" s="18" t="s">
+      <c r="V2" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
-      <c r="Y2" s="30"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="35"/>
       <c r="Z2" s="15"/>
-      <c r="AA2" s="18" t="s">
+      <c r="AA2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="AB2" s="19"/>
-      <c r="AC2" s="19"/>
-      <c r="AD2" s="19"/>
-      <c r="AE2" s="19"/>
-      <c r="AF2" s="19"/>
-      <c r="AG2" s="30"/>
+      <c r="AB2" s="24"/>
+      <c r="AC2" s="24"/>
+      <c r="AD2" s="24"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="35"/>
       <c r="AH2" s="16"/>
-      <c r="AI2" s="18" t="s">
+      <c r="AI2" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="AJ2" s="19"/>
-      <c r="AK2" s="19"/>
-      <c r="AL2" s="19"/>
-      <c r="AM2" s="19"/>
-      <c r="AN2" s="19"/>
-      <c r="AO2" s="19"/>
-      <c r="AP2" s="19"/>
+      <c r="AJ2" s="24"/>
+      <c r="AK2" s="24"/>
+      <c r="AL2" s="24"/>
+      <c r="AM2" s="24"/>
+      <c r="AN2" s="24"/>
+      <c r="AO2" s="24"/>
+      <c r="AP2" s="24"/>
     </row>
     <row r="3" spans="2:67" s="8" customFormat="1" ht="40" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="30" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="17" t="s">
@@ -1174,12 +1187,12 @@
       <c r="AA3" s="7"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="22"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -1362,522 +1375,522 @@
       </c>
     </row>
     <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="19">
         <v>0</v>
       </c>
-      <c r="D5" s="32">
+      <c r="D5" s="19">
         <v>0</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="19">
         <v>0</v>
       </c>
-      <c r="F5" s="32">
+      <c r="F5" s="19">
         <v>0</v>
       </c>
-      <c r="G5" s="33">
+      <c r="G5" s="20">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="19">
         <v>21</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="19">
         <v>2</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="19">
+        <v>19</v>
+      </c>
+      <c r="F6" s="19">
+        <v>1</v>
+      </c>
+      <c r="G6" s="20">
         <v>0</v>
       </c>
-      <c r="F6" s="32">
+    </row>
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="19">
+        <v>20</v>
+      </c>
+      <c r="D7" s="19">
+        <v>1</v>
+      </c>
+      <c r="E7" s="19">
+        <v>18</v>
+      </c>
+      <c r="F7" s="19">
+        <v>2</v>
+      </c>
+      <c r="G7" s="20">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="19">
+        <v>25</v>
+      </c>
+      <c r="D8" s="19">
+        <v>5</v>
+      </c>
+      <c r="E8" s="19">
         <v>0</v>
       </c>
-      <c r="G6" s="33">
+      <c r="F8" s="19">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="32">
+      <c r="G8" s="20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="19">
+        <v>26</v>
+      </c>
+      <c r="D9" s="19">
+        <v>7</v>
+      </c>
+      <c r="E9" s="19">
+        <v>19</v>
+      </c>
+      <c r="F9" s="19">
+        <v>4</v>
+      </c>
+      <c r="G9" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="19">
+        <v>1</v>
+      </c>
+      <c r="D10" s="19">
+        <v>1</v>
+      </c>
+      <c r="E10" s="19">
+        <v>1</v>
+      </c>
+      <c r="F10" s="19">
+        <v>1</v>
+      </c>
+      <c r="G10" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="19">
+        <v>1</v>
+      </c>
+      <c r="D11" s="19">
+        <v>4</v>
+      </c>
+      <c r="E11" s="19">
+        <v>1</v>
+      </c>
+      <c r="F11" s="19">
+        <v>17</v>
+      </c>
+      <c r="G11" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="19">
+        <v>1</v>
+      </c>
+      <c r="D12" s="19">
+        <v>2</v>
+      </c>
+      <c r="E12" s="19">
+        <v>1</v>
+      </c>
+      <c r="F12" s="19">
+        <v>2</v>
+      </c>
+      <c r="G12" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="19">
+        <v>1</v>
+      </c>
+      <c r="D13" s="19">
+        <v>7</v>
+      </c>
+      <c r="E13" s="19">
+        <v>1</v>
+      </c>
+      <c r="F13" s="19">
+        <v>18</v>
+      </c>
+      <c r="G13" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="19">
+        <v>2</v>
+      </c>
+      <c r="D14" s="19">
+        <v>2</v>
+      </c>
+      <c r="E14" s="19">
+        <v>2</v>
+      </c>
+      <c r="F14" s="19">
+        <v>1</v>
+      </c>
+      <c r="G14" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="21">
+        <v>3</v>
+      </c>
+      <c r="D15" s="19">
+        <v>3</v>
+      </c>
+      <c r="E15" s="19">
+        <v>3</v>
+      </c>
+      <c r="F15" s="19">
+        <v>1</v>
+      </c>
+      <c r="G15" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="19">
+        <v>4</v>
+      </c>
+      <c r="D16" s="19">
+        <v>3</v>
+      </c>
+      <c r="E16" s="19">
+        <v>3</v>
+      </c>
+      <c r="F16" s="19">
+        <v>1</v>
+      </c>
+      <c r="G16" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="19">
+        <v>4</v>
+      </c>
+      <c r="D17" s="19">
+        <v>3</v>
+      </c>
+      <c r="E17" s="19">
+        <v>3</v>
+      </c>
+      <c r="F17" s="19">
+        <v>1</v>
+      </c>
+      <c r="G17" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="19">
+        <v>4</v>
+      </c>
+      <c r="D18" s="19">
+        <v>2</v>
+      </c>
+      <c r="E18" s="19">
+        <v>3</v>
+      </c>
+      <c r="F18" s="19">
+        <v>1</v>
+      </c>
+      <c r="G18" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="19">
+        <v>5</v>
+      </c>
+      <c r="D19" s="19">
+        <v>5</v>
+      </c>
+      <c r="E19" s="19">
+        <v>3</v>
+      </c>
+      <c r="F19" s="19">
+        <v>4</v>
+      </c>
+      <c r="G19" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="32">
-        <v>1</v>
-      </c>
-      <c r="E7" s="32">
-        <v>18</v>
-      </c>
-      <c r="F7" s="32">
-        <v>0</v>
-      </c>
-      <c r="G7" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="32">
+      <c r="C20" s="19">
+        <v>3</v>
+      </c>
+      <c r="D20" s="19">
+        <v>3</v>
+      </c>
+      <c r="E20" s="19">
+        <v>4</v>
+      </c>
+      <c r="F20" s="19">
+        <v>2</v>
+      </c>
+      <c r="G20" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="32">
+      <c r="C21" s="19">
+        <v>4</v>
+      </c>
+      <c r="D21" s="19">
+        <v>4</v>
+      </c>
+      <c r="E21" s="19">
+        <v>4</v>
+      </c>
+      <c r="F21" s="19">
+        <v>1</v>
+      </c>
+      <c r="G21" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="19">
+        <v>4</v>
+      </c>
+      <c r="D22" s="19">
+        <v>4</v>
+      </c>
+      <c r="E22" s="19">
         <v>5</v>
       </c>
-      <c r="E8" s="32">
-        <v>0</v>
-      </c>
-      <c r="F8" s="32">
-        <v>0</v>
-      </c>
-      <c r="G8" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="32">
-        <v>26</v>
-      </c>
-      <c r="D9" s="32">
+      <c r="F22" s="19">
+        <v>2</v>
+      </c>
+      <c r="G22" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="19">
         <v>7</v>
       </c>
-      <c r="E9" s="32">
-        <v>0</v>
-      </c>
-      <c r="F9" s="32">
-        <v>0</v>
-      </c>
-      <c r="G9" s="33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="35" t="s">
+      <c r="D23" s="19">
+        <v>2</v>
+      </c>
+      <c r="E23" s="19">
+        <v>10</v>
+      </c>
+      <c r="F23" s="19">
+        <v>1</v>
+      </c>
+      <c r="G23" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="19">
+        <v>21</v>
+      </c>
+      <c r="D24" s="19">
+        <v>2</v>
+      </c>
+      <c r="E24" s="19">
+        <v>10</v>
+      </c>
+      <c r="F24" s="19">
+        <v>1</v>
+      </c>
+      <c r="G24" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="19">
+        <v>11</v>
+      </c>
+      <c r="D25" s="19">
+        <v>1</v>
+      </c>
+      <c r="E25" s="19">
+        <v>11</v>
+      </c>
+      <c r="F25" s="19">
+        <v>1</v>
+      </c>
+      <c r="G25" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="19">
         <v>15</v>
       </c>
-      <c r="C10" s="32">
-        <v>1</v>
-      </c>
-      <c r="D10" s="32">
-        <v>1</v>
-      </c>
-      <c r="E10" s="32">
-        <v>1</v>
-      </c>
-      <c r="F10" s="32">
-        <v>1</v>
-      </c>
-      <c r="G10" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="32">
-        <v>1</v>
-      </c>
-      <c r="D11" s="32">
-        <v>4</v>
-      </c>
-      <c r="E11" s="32">
-        <v>1</v>
-      </c>
-      <c r="F11" s="32">
+      <c r="D26" s="19">
+        <v>3</v>
+      </c>
+      <c r="E26" s="19">
+        <v>15</v>
+      </c>
+      <c r="F26" s="19">
+        <v>3</v>
+      </c>
+      <c r="G26" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="19">
+        <v>11</v>
+      </c>
+      <c r="D27" s="19">
+        <v>2</v>
+      </c>
+      <c r="E27" s="19">
+        <v>16</v>
+      </c>
+      <c r="F27" s="19">
+        <v>1</v>
+      </c>
+      <c r="G27" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="19">
+        <v>12</v>
+      </c>
+      <c r="D28" s="19">
+        <v>2</v>
+      </c>
+      <c r="E28" s="19">
+        <v>16</v>
+      </c>
+      <c r="F28" s="19">
+        <v>1</v>
+      </c>
+      <c r="G28" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="19">
+        <v>22</v>
+      </c>
+      <c r="D29" s="19">
+        <v>2</v>
+      </c>
+      <c r="E29" s="19">
+        <v>16</v>
+      </c>
+      <c r="F29" s="19">
+        <v>1</v>
+      </c>
+      <c r="G29" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="19">
+        <v>7</v>
+      </c>
+      <c r="D30" s="19">
+        <v>7</v>
+      </c>
+      <c r="E30" s="19">
         <v>17</v>
       </c>
-      <c r="G11" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="32">
-        <v>1</v>
-      </c>
-      <c r="D12" s="32">
+      <c r="F30" s="19">
         <v>2</v>
       </c>
-      <c r="E12" s="32">
-        <v>1</v>
-      </c>
-      <c r="F12" s="32">
-        <v>2</v>
-      </c>
-      <c r="G12" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="32">
-        <v>1</v>
-      </c>
-      <c r="D13" s="32">
-        <v>7</v>
-      </c>
-      <c r="E13" s="32">
-        <v>1</v>
-      </c>
-      <c r="F13" s="32">
-        <v>18</v>
-      </c>
-      <c r="G13" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="32">
-        <v>2</v>
-      </c>
-      <c r="D14" s="32">
-        <v>2</v>
-      </c>
-      <c r="E14" s="32">
-        <v>2</v>
-      </c>
-      <c r="F14" s="32">
-        <v>1</v>
-      </c>
-      <c r="G14" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="34">
-        <v>3</v>
-      </c>
-      <c r="D15" s="32">
-        <v>3</v>
-      </c>
-      <c r="E15" s="32">
-        <v>3</v>
-      </c>
-      <c r="F15" s="32">
-        <v>1</v>
-      </c>
-      <c r="G15" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="35" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="32">
-        <v>4</v>
-      </c>
-      <c r="D16" s="32">
-        <v>3</v>
-      </c>
-      <c r="E16" s="32">
-        <v>3</v>
-      </c>
-      <c r="F16" s="32">
-        <v>1</v>
-      </c>
-      <c r="G16" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="32">
-        <v>4</v>
-      </c>
-      <c r="D17" s="32">
-        <v>3</v>
-      </c>
-      <c r="E17" s="32">
-        <v>3</v>
-      </c>
-      <c r="F17" s="32">
-        <v>1</v>
-      </c>
-      <c r="G17" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="32">
-        <v>4</v>
-      </c>
-      <c r="D18" s="32">
-        <v>2</v>
-      </c>
-      <c r="E18" s="32">
-        <v>3</v>
-      </c>
-      <c r="F18" s="32">
-        <v>1</v>
-      </c>
-      <c r="G18" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="32">
-        <v>5</v>
-      </c>
-      <c r="D19" s="32">
-        <v>5</v>
-      </c>
-      <c r="E19" s="32">
-        <v>3</v>
-      </c>
-      <c r="F19" s="32">
-        <v>4</v>
-      </c>
-      <c r="G19" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="35" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="32">
-        <v>3</v>
-      </c>
-      <c r="D20" s="32">
-        <v>3</v>
-      </c>
-      <c r="E20" s="32">
-        <v>4</v>
-      </c>
-      <c r="F20" s="32">
-        <v>2</v>
-      </c>
-      <c r="G20" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="32">
-        <v>4</v>
-      </c>
-      <c r="D21" s="32">
-        <v>4</v>
-      </c>
-      <c r="E21" s="32">
-        <v>4</v>
-      </c>
-      <c r="F21" s="32">
-        <v>1</v>
-      </c>
-      <c r="G21" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="35" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="32">
-        <v>4</v>
-      </c>
-      <c r="D22" s="32">
-        <v>4</v>
-      </c>
-      <c r="E22" s="32">
-        <v>5</v>
-      </c>
-      <c r="F22" s="32">
-        <v>2</v>
-      </c>
-      <c r="G22" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="35" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" s="32">
-        <v>7</v>
-      </c>
-      <c r="D23" s="32">
-        <v>2</v>
-      </c>
-      <c r="E23" s="32">
-        <v>10</v>
-      </c>
-      <c r="F23" s="32">
-        <v>1</v>
-      </c>
-      <c r="G23" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="32">
-        <v>21</v>
-      </c>
-      <c r="D24" s="32">
-        <v>2</v>
-      </c>
-      <c r="E24" s="32">
-        <v>10</v>
-      </c>
-      <c r="F24" s="32">
-        <v>1</v>
-      </c>
-      <c r="G24" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="35" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="32">
-        <v>11</v>
-      </c>
-      <c r="D25" s="32">
-        <v>1</v>
-      </c>
-      <c r="E25" s="32">
-        <v>11</v>
-      </c>
-      <c r="F25" s="32">
-        <v>1</v>
-      </c>
-      <c r="G25" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="35" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26" s="32">
-        <v>15</v>
-      </c>
-      <c r="D26" s="32">
-        <v>3</v>
-      </c>
-      <c r="E26" s="32">
-        <v>15</v>
-      </c>
-      <c r="F26" s="32">
-        <v>3</v>
-      </c>
-      <c r="G26" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="C27" s="32">
-        <v>11</v>
-      </c>
-      <c r="D27" s="32">
-        <v>2</v>
-      </c>
-      <c r="E27" s="32">
-        <v>16</v>
-      </c>
-      <c r="F27" s="32">
-        <v>1</v>
-      </c>
-      <c r="G27" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" s="32">
-        <v>12</v>
-      </c>
-      <c r="D28" s="32">
-        <v>2</v>
-      </c>
-      <c r="E28" s="32">
-        <v>16</v>
-      </c>
-      <c r="F28" s="32">
-        <v>1</v>
-      </c>
-      <c r="G28" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="C29" s="32">
-        <v>22</v>
-      </c>
-      <c r="D29" s="32">
-        <v>2</v>
-      </c>
-      <c r="E29" s="32">
-        <v>16</v>
-      </c>
-      <c r="F29" s="32">
-        <v>1</v>
-      </c>
-      <c r="G29" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30" s="32">
-        <v>7</v>
-      </c>
-      <c r="D30" s="32">
-        <v>7</v>
-      </c>
-      <c r="E30" s="32">
-        <v>17</v>
-      </c>
-      <c r="F30" s="32">
-        <v>2</v>
-      </c>
-      <c r="G30" s="33">
+      <c r="G30" s="20">
         <v>1</v>
       </c>
     </row>

</xml_diff>